<commit_message>
[dnn-library] [SW-3899] Lib Api: add custom impl selection for transformation node
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="15"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="69"/>
   </bookViews>
   <sheets>
     <sheet name="INFORMATION" sheetId="1" state="visible" r:id="rId2"/>
@@ -91,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2421" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2432" uniqueCount="95">
   <si>
     <t xml:space="preserve">There is one sheet per operator</t>
   </si>
@@ -12019,7 +12019,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:Q4"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
@@ -12054,6 +12054,12 @@
       <c r="K1" s="3"/>
       <c r="L1" s="3"/>
       <c r="M1" s="3"/>
+      <c r="N1" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -12093,6 +12099,18 @@
       <c r="M2" s="4" t="s">
         <v>8</v>
       </c>
+      <c r="N2" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="O2" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="P2" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q2" s="7" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -12134,6 +12152,18 @@
       <c r="M3" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="N3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q3" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -12175,13 +12205,26 @@
       <c r="M4" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="N4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q4" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="F1:I1"/>
     <mergeCell ref="J1:M1"/>
+    <mergeCell ref="N1:Q1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -12203,7 +12246,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="13.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="13.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="6" style="0" width="8.67"/>
   </cols>
   <sheetData>
@@ -12292,11 +12335,11 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="13.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="13.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="0" width="13.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="0" width="13.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="0" width="13.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="0" width="13.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="14" style="0" width="8.67"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
[dnn-library] restoring elementExp threaded implementation, as it was removed probably by mistake from the excel
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="9"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="22"/>
   </bookViews>
   <sheets>
     <sheet name="INFORMATION" sheetId="1" state="visible" r:id="rId2"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2443" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2454" uniqueCount="96">
   <si>
     <t xml:space="preserve">There is one sheet per operator</t>
   </si>
@@ -3102,7 +3102,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19"/>
@@ -3121,6 +3121,12 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
+      <c r="F1" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -3136,6 +3142,18 @@
       <c r="E2" s="4" t="s">
         <v>8</v>
       </c>
+      <c r="F2" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -3153,6 +3171,18 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -3170,11 +3200,25 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-    </row>
+      <c r="F4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
+    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4176] [SW-4117] Cleaning up non-optimized generic versions of element single instructions
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="20"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="68"/>
   </bookViews>
   <sheets>
     <sheet name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId2"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2314" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2248" uniqueCount="96">
   <si>
     <t xml:space="preserve">ET_adaptiveavgpool</t>
   </si>
@@ -2909,7 +2909,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19"/>
@@ -2928,12 +2928,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -2949,18 +2943,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -2978,18 +2960,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -3007,25 +2977,16 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -3042,7 +3003,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.98"/>
@@ -3063,12 +3024,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -3084,18 +3039,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -3113,18 +3056,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -3142,24 +3073,19 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -3176,7 +3102,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19"/>
@@ -3199,18 +3125,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -3226,30 +3140,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -3267,30 +3157,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -3308,37 +3174,17 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M4" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="J1:M1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -9867,7 +9713,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
@@ -9888,12 +9734,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -9909,18 +9749,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -9938,18 +9766,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -9967,24 +9783,16 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -11199,7 +11007,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.02"/>
@@ -11220,12 +11028,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -11241,18 +11043,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -11270,18 +11060,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -11299,24 +11077,16 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4133] Remove least optimized implementations for the Splat operator
Kept vectorized version as it is supposed to be generic
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="68"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="66"/>
   </bookViews>
   <sheets>
     <sheet name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId2"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2248" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2232" uniqueCount="96">
   <si>
     <t xml:space="preserve">ET_adaptiveavgpool</t>
   </si>
@@ -10781,7 +10781,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="14.01"/>
@@ -10803,18 +10803,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -10830,30 +10818,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -10871,37 +10835,19 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="J1:M1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4134] Cleaning up implementations of tensor view just keeping the most optimized generic version (vectorized) and removing the scalar and threaded versions
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="71"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="69"/>
   </bookViews>
   <sheets>
     <sheet name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId2"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2163" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2141" uniqueCount="96">
   <si>
     <t xml:space="preserve">ET_adaptiveavgpool</t>
   </si>
@@ -11064,7 +11064,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19"/>
@@ -11087,18 +11087,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -11114,30 +11102,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -11155,30 +11119,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -11196,37 +11136,20 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M4" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="J1:M1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4130] Remove least optimized implementations for the RowwiseQuantizedSparseLengthsWeightedSum operator
keeping scalar, removing threaded (as it supports the same cases as the vectorized one)
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="69"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="57"/>
   </bookViews>
   <sheets>
     <sheet name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId2"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2141" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2115" uniqueCount="96">
   <si>
     <t xml:space="preserve">ET_adaptiveavgpool</t>
   </si>
@@ -9046,7 +9046,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="49"/>
@@ -9070,17 +9070,11 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="6" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
-      <c r="J1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -9108,18 +9102,6 @@
       <c r="I2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -9149,18 +9131,6 @@
       <c r="I3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -9190,18 +9160,6 @@
       <c r="I4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -9231,18 +9189,6 @@
       <c r="I5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M5" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
@@ -9272,18 +9218,6 @@
       <c r="I6" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M6" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
@@ -9313,18 +9247,6 @@
       <c r="I7" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M7" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
@@ -9354,18 +9276,6 @@
       <c r="I8" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M8" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
@@ -9395,25 +9305,21 @@
       <c r="I9" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J9" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L9" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M9" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="F1:I1"/>
-    <mergeCell ref="J1:M1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4129] Remove least optimized implementations for the RowwiseQuantizedFullyConnected operator keeping vectorized as generic, aligned32B as optimized special case
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="57"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="56"/>
   </bookViews>
   <sheets>
     <sheet name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId2"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2115" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2069" uniqueCount="96">
   <si>
     <t xml:space="preserve">ET_adaptiveavgpool</t>
   </si>
@@ -8610,7 +8610,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="39.01"/>
@@ -8636,23 +8636,11 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="6" t="s">
-        <v>11</v>
+        <v>70</v>
       </c>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
-      <c r="J1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="O1" s="6"/>
-      <c r="P1" s="6"/>
-      <c r="Q1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -8680,30 +8668,6 @@
       <c r="I2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="N2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="O2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="P2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q2" s="7" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -8733,30 +8697,6 @@
       <c r="I3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="Q3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -8786,30 +8726,6 @@
       <c r="I4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="Q4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -8839,30 +8755,6 @@
       <c r="I5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="O5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="Q5" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
@@ -8892,30 +8784,6 @@
       <c r="I6" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="Q6" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
@@ -8945,30 +8813,6 @@
       <c r="I7" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M7" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="O7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="P7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="Q7" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
@@ -8998,38 +8842,13 @@
       <c r="I8" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M8" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="P8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="Q8" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="3">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="F1:I1"/>
-    <mergeCell ref="J1:M1"/>
-    <mergeCell ref="N1:Q1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4124] [SW-4125] Remove least optimized implementations for the FusedRowwiseQuantizedSparse* ops vectorized is generic?so just keeping that one
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="56"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="35"/>
   </bookViews>
   <sheets>
     <sheet name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId2"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2069" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1995" uniqueCount="96">
   <si>
     <t xml:space="preserve">ET_adaptiveavgpool</t>
   </si>
@@ -5039,7 +5039,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="45.98"/>
@@ -5062,18 +5062,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -5089,30 +5077,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -5130,30 +5094,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -5171,30 +5111,6 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -5212,30 +5128,6 @@
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M5" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
@@ -5253,37 +5145,13 @@
       <c r="E6" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M6" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="J1:M1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -5300,7 +5168,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="53.99"/>
@@ -5323,18 +5191,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -5350,30 +5206,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -5391,30 +5223,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -5432,30 +5240,6 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -5473,30 +5257,6 @@
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M5" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
@@ -5514,30 +5274,6 @@
       <c r="E6" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M6" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
@@ -5555,37 +5291,15 @@
       <c r="E7" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I7" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M7" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="J1:M1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4126] Remove least optimized implementations for the LocalResponseNormalization operator
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="35"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="45"/>
   </bookViews>
   <sheets>
     <sheet name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId2"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1995" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1981" uniqueCount="96">
   <si>
     <t xml:space="preserve">ET_adaptiveavgpool</t>
   </si>
@@ -6606,7 +6606,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="35"/>
@@ -6630,17 +6630,11 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="6" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
-      <c r="J1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -6668,18 +6662,6 @@
       <c r="I2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -6709,18 +6691,6 @@
       <c r="I3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -6750,18 +6720,6 @@
       <c r="I4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -6791,25 +6749,18 @@
       <c r="I5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M5" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="F1:I1"/>
-    <mergeCell ref="J1:M1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4123] Remove least optimized implementations for the FullyConnected operator vectorized appears to be generic => keeping only this one
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="45"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="34"/>
   </bookViews>
   <sheets>
     <sheet name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId2"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1981" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1947" uniqueCount="96">
   <si>
     <t xml:space="preserve">ET_adaptiveavgpool</t>
   </si>
@@ -4778,7 +4778,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.01"/>
@@ -4801,18 +4801,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -4828,30 +4816,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -4869,30 +4833,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -4910,30 +4850,6 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -4951,30 +4867,6 @@
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M5" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
@@ -4992,37 +4884,11 @@
       <c r="E6" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M6" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="J1:M1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4096] Remove scalar Convolution implementation removed scalar, keeping threaded (which can be removed once SW-3816 is fixed) as generic  and vectorized as the optimized one,.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="34"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="10"/>
   </bookViews>
   <sheets>
     <sheet name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId2"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1947" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1930" uniqueCount="96">
   <si>
     <t xml:space="preserve">ET_adaptiveavgpool</t>
   </si>
@@ -807,7 +807,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19.99"/>
@@ -831,17 +831,11 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="6" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
-      <c r="J1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -869,18 +863,6 @@
       <c r="I2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -910,18 +892,6 @@
       <c r="I3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -951,18 +921,6 @@
       <c r="I4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -992,18 +950,6 @@
       <c r="I5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M5" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
@@ -1033,25 +979,13 @@
       <c r="I6" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M6" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="F1:I1"/>
-    <mergeCell ref="J1:M1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4127] Remove least optimized implementations for the MatMul operator keeping just the vectorized (and vectorized transposed) version, as it is supposed to be generic.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="10"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="46"/>
   </bookViews>
   <sheets>
     <sheet name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId2"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1930" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1880" uniqueCount="94">
   <si>
     <t xml:space="preserve">ET_adaptiveavgpool</t>
   </si>
@@ -185,12 +185,6 @@
   </si>
   <si>
     <t xml:space="preserve">Tensorized</t>
-  </si>
-  <si>
-    <t xml:space="preserve">clean</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dirty</t>
   </si>
   <si>
     <t xml:space="preserve">ET_crossentropyloss</t>
@@ -1317,7 +1311,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.02"/>
@@ -1336,23 +1330,11 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="6" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
-      <c r="J1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="O1" s="6"/>
-      <c r="P1" s="6"/>
-      <c r="Q1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -1380,30 +1362,6 @@
       <c r="I2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="N2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="O2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="P2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q2" s="7" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -1433,30 +1391,6 @@
       <c r="I3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -1486,38 +1420,20 @@
       <c r="I4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q4" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="3">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="F1:I1"/>
-    <mergeCell ref="J1:M1"/>
-    <mergeCell ref="N1:Q1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -1547,7 +1463,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -1708,7 +1624,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -1799,7 +1715,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -1933,7 +1849,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -2098,7 +2014,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -2355,7 +2271,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -2521,7 +2437,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -2685,7 +2601,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -2846,7 +2762,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -2942,7 +2858,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -3043,7 +2959,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -3140,7 +3056,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -3303,7 +3219,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -3466,7 +3382,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -3629,7 +3545,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -3926,7 +3842,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -4118,7 +4034,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -4281,7 +4197,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -4502,7 +4418,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -4634,7 +4550,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -4727,7 +4643,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -4854,7 +4770,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -4983,7 +4899,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -5129,7 +5045,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -5292,7 +5208,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -5365,7 +5281,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>7</v>
@@ -5647,7 +5563,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -5779,7 +5695,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -5870,7 +5786,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -6031,7 +5947,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -6122,7 +6038,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -6285,7 +6201,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -6421,7 +6337,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -6494,7 +6410,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>7</v>
@@ -6577,7 +6493,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15"/>
@@ -6592,7 +6508,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -6600,18 +6516,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -6627,30 +6531,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -6668,30 +6548,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -6709,30 +6565,6 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -6750,37 +6582,20 @@
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="M5" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="J1:M1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -6810,7 +6625,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -6944,7 +6759,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -7017,7 +6832,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>7</v>
@@ -7245,7 +7060,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -7254,7 +7069,7 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
@@ -7385,7 +7200,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -7517,7 +7332,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -7560,7 +7375,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>7</v>
@@ -7642,7 +7457,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -7776,7 +7591,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -7908,7 +7723,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -7997,7 +7812,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -8092,7 +7907,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -8101,7 +7916,7 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
@@ -8345,7 +8160,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -8631,7 +8446,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -8828,7 +8643,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -8926,7 +8741,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -9064,7 +8879,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -9153,7 +8968,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -9276,7 +9091,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -9420,7 +9235,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -9586,7 +9401,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -9808,7 +9623,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -9888,7 +9703,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -9979,7 +9794,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -10269,7 +10084,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -10369,7 +10184,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -10442,7 +10257,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>7</v>
@@ -10534,7 +10349,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -10543,7 +10358,7 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
@@ -10663,17 +10478,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[dnn-library] [SW-4201] Restoring threaded version for fullyconnected as base implementation
some sparseNN tests with -O0 fail if using the vectorized version as base implementation.
Created SW-4213 to fix this
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="46"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="34"/>
   </bookViews>
   <sheets>
     <sheet name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId2"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1880" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1897" uniqueCount="94">
   <si>
     <t xml:space="preserve">ET_adaptiveavgpool</t>
   </si>
@@ -4628,7 +4628,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.01"/>
@@ -4651,6 +4651,12 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
+      <c r="F1" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -4666,6 +4672,18 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
+      <c r="F2" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -4683,6 +4701,18 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -4700,6 +4730,18 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -4717,6 +4759,18 @@
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
@@ -4734,11 +4788,24 @@
       <c r="E6" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="F6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
+    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>

<commit_message>
[dnn-library] restoring cross references between sheets
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="34"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId2"/>
@@ -974,7 +974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:A2"/>
@@ -1421,14 +1421,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:A2"/>
@@ -4929,8 +4929,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
@@ -5075,10 +5075,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
@@ -6533,12 +6533,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:A2"/>
@@ -6650,15 +6650,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
@@ -7227,12 +7227,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:A2"/>
@@ -8190,7 +8190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:A2"/>
@@ -8472,15 +8472,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:A2"/>
@@ -9431,9 +9431,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:A2"/>
@@ -9965,12 +9965,12 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -9986,16 +9986,16 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
+      <c r="F2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="I2" s="4" t="s">
         <v>5</v>
       </c>
     </row>
@@ -10209,15 +10209,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>

</xml_diff>

<commit_message>
[dnn-library] restoring copy cache state table (removed by error)
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="13"/>
   </bookViews>
   <sheets>
     <sheet name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId2"/>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1897" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1897" uniqueCount="96">
   <si>
     <t xml:space="preserve">ET_adaptiveavgpool</t>
   </si>
@@ -185,6 +185,12 @@
   </si>
   <si>
     <t xml:space="preserve">Tensorized</t>
+  </si>
+  <si>
+    <t xml:space="preserve">clean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dirty</t>
   </si>
   <si>
     <t xml:space="preserve">ET_crossentropyloss</t>
@@ -1380,13 +1386,13 @@
         <v>0</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="I3" s="1" t="n">
         <v>0</v>
@@ -1409,13 +1415,13 @@
         <v>0</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="I4" s="1" t="n">
         <v>0</v>
@@ -1463,7 +1469,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -1624,7 +1630,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -1715,7 +1721,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -1849,7 +1855,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -2014,7 +2020,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -2271,7 +2277,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -2437,7 +2443,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -2601,7 +2607,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -2762,7 +2768,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -2858,7 +2864,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -2959,7 +2965,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -3056,7 +3062,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -3219,7 +3225,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -3382,7 +3388,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -3545,7 +3551,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -3842,7 +3848,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -4034,7 +4040,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -4197,7 +4203,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -4418,7 +4424,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -4550,7 +4556,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -4643,7 +4649,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -4837,7 +4843,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -4966,7 +4972,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -5112,7 +5118,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -5275,7 +5281,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -5348,7 +5354,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>7</v>
@@ -5630,7 +5636,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -5762,7 +5768,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -5853,7 +5859,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -6014,7 +6020,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -6105,7 +6111,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -6268,7 +6274,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -6404,7 +6410,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -6477,7 +6483,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>7</v>
@@ -6575,7 +6581,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -6692,7 +6698,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -6826,7 +6832,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -6899,7 +6905,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>7</v>
@@ -7127,7 +7133,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -7136,7 +7142,7 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
@@ -7267,7 +7273,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -7399,7 +7405,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -7442,7 +7448,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>7</v>
@@ -7524,7 +7530,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -7658,7 +7664,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -7790,7 +7796,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -7879,7 +7885,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -7974,7 +7980,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -7983,7 +7989,7 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
@@ -8227,7 +8233,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -8513,7 +8519,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -8710,7 +8716,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -8808,7 +8814,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -8946,7 +8952,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -9035,7 +9041,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -9158,7 +9164,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -9302,7 +9308,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -9468,7 +9474,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -9690,7 +9696,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -9770,7 +9776,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -9861,7 +9867,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -10151,7 +10157,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -10251,7 +10257,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -10324,7 +10330,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>7</v>
@@ -10416,7 +10422,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -10425,7 +10431,7 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
@@ -10545,17 +10551,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[dnn-library] [SW-4235] Operator Modulo has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -9317,7 +9317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="8" width="15"/>
@@ -9339,11 +9339,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="13" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="9">
       <c r="B2" s="12" t="inlineStr">
@@ -9366,26 +9361,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="14" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="14" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="14" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="9">
       <c r="A3" s="10" t="inlineStr">
@@ -9411,24 +9386,6 @@
       <c r="E3" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="9">
       <c r="A4" s="10" t="inlineStr">
@@ -9452,24 +9409,6 @@
         </is>
       </c>
       <c r="E4" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12817,7 +12756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="8" width="19.99"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4232] Operator LengthsSum has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -7804,7 +7804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="8" width="19"/>
@@ -7826,11 +7826,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="13" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="9">
       <c r="B2" s="12" t="inlineStr">
@@ -7853,26 +7848,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="14" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="14" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="14" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="9">
       <c r="A3" s="10" t="inlineStr">
@@ -7898,24 +7873,6 @@
       <c r="E3" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="9">
       <c r="A4" s="10" t="inlineStr">
@@ -7941,24 +7898,6 @@
       <c r="E4" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="8" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="5" s="9">
       <c r="A5" s="10" t="inlineStr">
@@ -7982,24 +7921,6 @@
         </is>
       </c>
       <c r="E5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I5" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9317,7 +9238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="8" width="15"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4223] Operator CrossEntropyLoss has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -1710,7 +1710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="8" width="25"/>
@@ -1732,11 +1732,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="13" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="9">
       <c r="B2" s="12" t="inlineStr">
@@ -1759,26 +1754,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="14" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="14" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="14" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="9">
       <c r="A3" s="10" t="inlineStr">
@@ -1804,24 +1779,6 @@
       <c r="E3" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="9">
       <c r="A4" s="10" t="inlineStr">
@@ -1847,24 +1804,6 @@
       <c r="E4" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="8" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="5" s="9">
       <c r="A5" s="10" t="inlineStr">
@@ -1888,24 +1827,6 @@
         </is>
       </c>
       <c r="E5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I5" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7804,7 +7725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="8" width="19"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4229] Operator GatherRanges has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -1710,7 +1710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="8" width="25"/>
@@ -6637,7 +6637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="8" width="20.98"/>
@@ -6659,11 +6659,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="13" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="9">
       <c r="B2" s="12" t="inlineStr">
@@ -6686,26 +6681,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="14" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="14" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="14" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="9">
       <c r="A3" s="10" t="inlineStr">
@@ -6731,24 +6706,6 @@
       <c r="E3" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="9">
       <c r="A4" s="10" t="inlineStr">
@@ -6774,24 +6731,6 @@
       <c r="E4" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="8" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="5" s="9">
       <c r="A5" s="10" t="inlineStr">
@@ -6817,24 +6756,6 @@
       <c r="E5" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I5" s="8" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="6" s="9">
       <c r="A6" s="10" t="inlineStr">
@@ -6858,24 +6779,6 @@
         </is>
       </c>
       <c r="E6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I6" s="8" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[dnn-library] [SW-4236] Operator Quantize has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -6637,7 +6637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="8" width="20.98"/>
@@ -9335,7 +9335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="8" width="17"/>
@@ -9357,11 +9357,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="13" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="9">
       <c r="B2" s="12" t="inlineStr">
@@ -9384,26 +9379,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="14" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="14" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="14" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="9">
       <c r="A3" s="10" t="inlineStr">
@@ -9429,24 +9404,6 @@
       <c r="E3" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="9">
       <c r="A4" s="10" t="inlineStr">
@@ -9470,24 +9427,6 @@
         </is>
       </c>
       <c r="E4" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="8" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[dnn-library] [SW-4221] Operator BatchedReduceAdd has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -7306,7 +7306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="23.01"/>
@@ -8631,7 +8631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="25"/>
@@ -8653,11 +8653,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="10">
       <c r="B2" s="13" t="inlineStr">
@@ -8680,26 +8675,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="10">
       <c r="A3" s="11" t="inlineStr">
@@ -8725,24 +8700,6 @@
       <c r="E3" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="10">
       <c r="A4" s="11" t="inlineStr">
@@ -8766,24 +8723,6 @@
         </is>
       </c>
       <c r="E4" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[dnn-library] [SW-4220] Operator BatchedAdd has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -6805,7 +6805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="19"/>
@@ -6827,11 +6827,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="10">
       <c r="B2" s="13" t="inlineStr">
@@ -6854,26 +6849,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="10">
       <c r="A3" s="11" t="inlineStr">
@@ -6899,24 +6874,6 @@
       <c r="E3" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="10">
       <c r="A4" s="11" t="inlineStr">
@@ -6942,24 +6899,6 @@
       <c r="E4" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="5" s="10">
       <c r="A5" s="11" t="inlineStr">
@@ -6983,24 +6922,6 @@
         </is>
       </c>
       <c r="E5" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I5" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8631,7 +8552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="25"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4226] Operator ExtractTensor has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5519,7 +5519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="22.01"/>
@@ -5541,11 +5541,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="10">
       <c r="B2" s="13" t="inlineStr">
@@ -5568,26 +5563,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="10">
       <c r="A3" s="11" t="inlineStr">
@@ -5613,24 +5588,6 @@
       <c r="E3" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="10">
       <c r="A4" s="11" t="inlineStr">
@@ -5654,24 +5611,6 @@
         </is>
       </c>
       <c r="E4" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6805,7 +6744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="19"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4228] Operator Gather has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5519,7 +5519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="22.01"/>
@@ -6363,7 +6363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="15"/>
@@ -6385,11 +6385,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="10">
       <c r="B2" s="13" t="inlineStr">
@@ -6412,26 +6407,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="10">
       <c r="A3" s="11" t="inlineStr">
@@ -6457,24 +6432,6 @@
       <c r="E3" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="10">
       <c r="A4" s="11" t="inlineStr">
@@ -6500,24 +6457,6 @@
       <c r="E4" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="5" s="10">
       <c r="A5" s="11" t="inlineStr">
@@ -6541,24 +6480,6 @@
         </is>
       </c>
       <c r="E5" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I5" s="9" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[dnn-library] [SW-4240] Operator SparseToDenseMask has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -6363,7 +6363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="15"/>
@@ -11579,7 +11579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="26"/>
@@ -11601,11 +11601,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="10">
       <c r="B2" s="13" t="inlineStr">
@@ -11628,26 +11623,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="10">
       <c r="A3" s="11" t="inlineStr">
@@ -11673,24 +11648,6 @@
       <c r="E3" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="10">
       <c r="A4" s="11" t="inlineStr">
@@ -11716,24 +11673,6 @@
       <c r="E4" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="5" s="10">
       <c r="A5" s="11" t="inlineStr">
@@ -11759,24 +11698,6 @@
       <c r="E5" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I5" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="6" s="10">
       <c r="A6" s="11" t="inlineStr">
@@ -11802,24 +11723,6 @@
       <c r="E6" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H6" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I6" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="7" s="10">
       <c r="A7" s="11" t="inlineStr">
@@ -11843,24 +11746,6 @@
         </is>
       </c>
       <c r="E7" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I7" s="9" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[dnn-library] [SW-4233] Operator LengthsToRanges has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -7474,7 +7474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="24"/>
@@ -7496,11 +7496,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="10">
       <c r="B2" s="13" t="inlineStr">
@@ -7523,26 +7518,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="10">
       <c r="A3" s="11" t="inlineStr">
@@ -7568,24 +7543,6 @@
       <c r="E3" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="10">
       <c r="A4" s="11" t="inlineStr">
@@ -7609,24 +7566,6 @@
         </is>
       </c>
       <c r="E4" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11579,7 +11518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="26"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4225] Operator ElementSelect has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -4739,7 +4739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="22.01"/>
@@ -4761,11 +4761,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="10">
       <c r="B2" s="13" t="inlineStr">
@@ -4788,26 +4783,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="10">
       <c r="A3" s="11" t="inlineStr">
@@ -4833,24 +4808,6 @@
       <c r="E3" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="10">
       <c r="A4" s="11" t="inlineStr">
@@ -4876,24 +4833,6 @@
       <c r="E4" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="5" s="10">
       <c r="A5" s="11" t="inlineStr">
@@ -4919,24 +4858,6 @@
       <c r="E5" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I5" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="6" s="10">
       <c r="A6" s="11" t="inlineStr">
@@ -4960,24 +4881,6 @@
         </is>
       </c>
       <c r="E6" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H6" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I6" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7474,7 +7377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="24"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4224] Operator Dequantize has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -1962,7 +1962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="19"/>
@@ -1984,11 +1984,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="10">
       <c r="B2" s="13" t="inlineStr">
@@ -2011,26 +2006,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="10">
       <c r="A3" s="11" t="inlineStr">
@@ -2056,24 +2031,6 @@
       <c r="E3" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="10">
       <c r="A4" s="11" t="inlineStr">
@@ -2097,24 +2054,6 @@
         </is>
       </c>
       <c r="E4" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4739,7 +4678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="22.01"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4222] Operator Convolution3D has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -1114,7 +1114,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="22.01"/>
@@ -1136,11 +1136,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="10">
       <c r="B2" s="13" t="inlineStr">
@@ -1163,26 +1158,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="10">
       <c r="A3" s="11" t="inlineStr">
@@ -1208,24 +1183,6 @@
       <c r="E3" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="10">
       <c r="A4" s="11" t="inlineStr">
@@ -1251,24 +1208,6 @@
       <c r="E4" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="5" s="10">
       <c r="A5" s="11" t="inlineStr">
@@ -1294,24 +1233,6 @@
       <c r="E5" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I5" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="6" s="10">
       <c r="A6" s="11" t="inlineStr">
@@ -1335,24 +1256,6 @@
         </is>
       </c>
       <c r="E6" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H6" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I6" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1962,7 +1865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="19"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4239] Operator SparseToDense has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -1114,7 +1114,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="22.01"/>
@@ -11041,7 +11041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="22.01"/>
@@ -11065,11 +11065,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
-        <is>
-          <t>Vectorized</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="10">
       <c r="B2" s="13" t="inlineStr">
@@ -11092,26 +11087,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="10">
       <c r="A3" s="11" t="inlineStr">
@@ -11137,24 +11112,6 @@
       <c r="E3" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="10">
       <c r="A4" s="11" t="inlineStr">
@@ -11180,24 +11137,6 @@
       <c r="E4" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="5" s="10">
       <c r="A5" s="11" t="inlineStr">
@@ -11221,24 +11160,6 @@
         </is>
       </c>
       <c r="E5" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I5" s="9" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[dnn-library] [SW-4237] Operator RescaleQuantized has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -8781,7 +8781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="25"/>
@@ -8803,11 +8803,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="10">
       <c r="B2" s="13" t="inlineStr">
@@ -8830,26 +8825,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="10">
       <c r="A3" s="11" t="inlineStr">
@@ -8875,24 +8850,6 @@
       <c r="E3" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="10">
       <c r="A4" s="11" t="inlineStr">
@@ -8916,24 +8873,6 @@
         </is>
       </c>
       <c r="E4" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11041,7 +10980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="22.01"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-4234] Operator MaxPool has multiple implementations and no custom impl selector [SW-4242] Operator MaxPoolWihtArgMax has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -7727,11 +7727,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="10">
       <c r="B2" s="13" t="inlineStr">
@@ -7754,26 +7749,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="10">
       <c r="A3" s="11" t="inlineStr">
@@ -7799,24 +7774,6 @@
       <c r="E3" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="10">
       <c r="A4" s="11" t="inlineStr">
@@ -7840,24 +7797,6 @@
         </is>
       </c>
       <c r="E4" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7879,7 +7818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="26"/>
@@ -7901,11 +7840,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="10">
       <c r="B2" s="13" t="inlineStr">
@@ -7928,26 +7862,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="10">
       <c r="A3" s="11" t="inlineStr">
@@ -7973,24 +7887,6 @@
       <c r="E3" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="10">
       <c r="A4" s="11" t="inlineStr">
@@ -8016,24 +7912,6 @@
       <c r="E4" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="5" s="10">
       <c r="A5" s="11" t="inlineStr">
@@ -8057,24 +7935,6 @@
         </is>
       </c>
       <c r="E5" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I5" s="9" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[dnn-library] [SW-4241] Operator TopK has multiple implementations and no custom impl selector
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -7818,7 +7818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="26"/>
@@ -11781,7 +11781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="13.02"/>
@@ -11803,11 +11803,6 @@
           <t>BaseImpl</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
-        <is>
-          <t>Threaded</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="2" s="10">
       <c r="B2" s="13" t="inlineStr">
@@ -11830,26 +11825,6 @@
           <t>evictAv</t>
         </is>
       </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="3" s="10">
       <c r="A3" s="11" t="inlineStr">
@@ -11875,24 +11850,6 @@
       <c r="E3" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="4" s="10">
       <c r="A4" s="11" t="inlineStr">
@@ -11918,24 +11875,6 @@
       <c r="E4" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row customHeight="1" ht="15" r="5" s="10">
       <c r="A5" s="11" t="inlineStr">
@@ -11959,24 +11898,6 @@
         </is>
       </c>
       <c r="E5" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I5" s="9" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[dnn-library] [SW-4523] lib manager scripts need to check compatibility with excel and sheet names longer than 31 chars
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -14,7 +14,7 @@
     <sheet name="ET_batchedreduceadd" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="ET_batchedreducemin" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="ET_batchonehot" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ET_channelwisequantizedconvolution" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="ET_channelwisequantizedconv" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="ET_checksum" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="ET_convertto" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="ET_convolution" sheetId="11" state="visible" r:id="rId11"/>
@@ -41,9 +41,9 @@
     <sheet name="ET_embeddingbag" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="ET_extracttensor" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="ET_flip" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="ET_fullyconnected" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="ET_fusedrowwisequantizedsparselengthssum" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="ET_fusedrowwisequantizedsparselengthsweightedsum" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="ET_frwquantizedsparselengthssum" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="ET_frwquantizedsparselwsum" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="ET_fullyconnected" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="ET_gather" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="ET_gatherranges" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="ET_inserttensor" sheetId="40" state="visible" r:id="rId40"/>
@@ -63,8 +63,8 @@
     <sheet name="ET_rescalequantized" sheetId="54" state="visible" r:id="rId54"/>
     <sheet name="ET_resizebilinear" sheetId="55" state="visible" r:id="rId55"/>
     <sheet name="ET_resizenearest" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet name="ET_rowwisequantizedfullyconnected" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet name="ET_rowwisequantizedsparselengthsweightedsum" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet name="ET_rwquantizedfullyconnected" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="ET_rwquantizedsparselengthswsum" sheetId="58" state="visible" r:id="rId58"/>
     <sheet name="ET_scatterdata" sheetId="59" state="visible" r:id="rId59"/>
     <sheet name="ET_sigmoid" sheetId="60" state="visible" r:id="rId60"/>
     <sheet name="ET_softmax" sheetId="61" state="visible" r:id="rId61"/>
@@ -5487,268 +5487,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
-  <cols>
-    <col customWidth="1" max="1" min="1" style="9" width="23.01"/>
-    <col customWidth="1" max="2" min="2" style="9" width="14.01"/>
-    <col customWidth="1" max="5" min="3" style="9" width="13.02"/>
-    <col customWidth="1" max="6" min="6" style="9" width="16"/>
-    <col customWidth="1" max="9" min="7" style="9" width="13.02"/>
-    <col customWidth="1" max="10" min="10" style="9" width="18"/>
-    <col customWidth="1" max="13" min="11" style="9" width="13.02"/>
-    <col customWidth="1" max="1025" min="14" style="9" width="8.67"/>
-  </cols>
-  <sheetData>
-    <row customHeight="1" ht="15" r="1" s="10">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>ET_fullyconnected</t>
-        </is>
-      </c>
-      <c r="B1" s="12" t="inlineStr">
-        <is>
-          <t>BaseImpl</t>
-        </is>
-      </c>
-      <c r="F1" s="14" t="inlineStr">
-        <is>
-          <t>Vectorized</t>
-        </is>
-      </c>
-    </row>
-    <row customHeight="1" ht="15" r="2" s="10">
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="C2" s="13" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="D2" s="13" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="E2" s="13" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
-    </row>
-    <row customHeight="1" ht="15" r="3" s="10">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>out0</t>
-        </is>
-      </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="15" r="4" s="10">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>in0</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="15" r="5" s="10">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>in1</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I5" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="15" r="6" s="10">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>in2</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="H6" s="9" t="inlineStr">
-        <is>
-          <t>invalid</t>
-        </is>
-      </c>
-      <c r="I6" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
-  </mergeCells>
-  <printOptions gridLines="0" gridLinesSet="1" headings="0" horizontalCentered="0" verticalCentered="0"/>
-  <pageMargins bottom="1" footer="0.511805555555555" header="0.511805555555555" left="0.75" right="0.75" top="1"/>
-  <pageSetup blackAndWhite="0" copies="1" draft="0" firstPageNumber="0" fitToHeight="1" fitToWidth="1" horizontalDpi="300" orientation="portrait" pageOrder="downThenOver" paperSize="1" scale="100" useFirstPageNumber="0" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
   <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
@@ -5909,7 +5647,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6095,6 +5833,268 @@
   <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
+  </mergeCells>
+  <printOptions gridLines="0" gridLinesSet="1" headings="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins bottom="1" footer="0.511805555555555" header="0.511805555555555" left="0.75" right="0.75" top="1"/>
+  <pageSetup blackAndWhite="0" copies="1" draft="0" firstPageNumber="0" fitToHeight="1" fitToWidth="1" horizontalDpi="300" orientation="portrait" pageOrder="downThenOver" paperSize="1" scale="100" useFirstPageNumber="0" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
+  <cols>
+    <col customWidth="1" max="1" min="1" style="9" width="23.01"/>
+    <col customWidth="1" max="2" min="2" style="9" width="14.01"/>
+    <col customWidth="1" max="5" min="3" style="9" width="13.02"/>
+    <col customWidth="1" max="6" min="6" style="9" width="16"/>
+    <col customWidth="1" max="9" min="7" style="9" width="13.02"/>
+    <col customWidth="1" max="10" min="10" style="9" width="18"/>
+    <col customWidth="1" max="13" min="11" style="9" width="13.02"/>
+    <col customWidth="1" max="1025" min="14" style="9" width="8.67"/>
+  </cols>
+  <sheetData>
+    <row customHeight="1" ht="15" r="1" s="10">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>ET_fullyconnected</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>BaseImpl</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>Vectorized</t>
+        </is>
+      </c>
+    </row>
+    <row customHeight="1" ht="15" r="2" s="10">
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t>evictAv</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="I2" s="15" t="inlineStr">
+        <is>
+          <t>evictAv</t>
+        </is>
+      </c>
+    </row>
+    <row customHeight="1" ht="15" r="3" s="10">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>out0</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row customHeight="1" ht="15" r="4" s="10">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>in0</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row customHeight="1" ht="15" r="5" s="10">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>in1</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row customHeight="1" ht="15" r="6" s="10">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>in2</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>invalid</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <printOptions gridLines="0" gridLinesSet="1" headings="0" horizontalCentered="0" verticalCentered="0"/>
   <pageMargins bottom="1" footer="0.511805555555555" header="0.511805555555555" left="0.75" right="0.75" top="1"/>
@@ -11781,7 +11781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0" zeroHeight="0"/>
   <cols>
     <col customWidth="1" max="1" min="1" style="9" width="13.02"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-5914] Remove scalar version of Embedding Bag in lib
 * removing scalar version in code
 * removing references in excel tables
 * regenerating api and include files
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="8"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="30"/>
   </bookViews>
   <sheets>
     <sheet name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId2"/>
@@ -91,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1602" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1582" uniqueCount="95">
   <si>
     <t xml:space="preserve">ET_adaptiveavgpool</t>
   </si>
@@ -3836,7 +3836,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.98"/>
@@ -3857,12 +3857,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -3878,18 +3872,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -3907,18 +3889,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -3936,18 +3906,6 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -3965,18 +3923,6 @@
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
@@ -3994,18 +3940,6 @@
       <c r="E6" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I6" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
@@ -4023,24 +3957,11 @@
       <c r="E7" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I7" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>

<commit_message>
[dnn-library] Updating ElementBinary to use generalized loops
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="30"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="29"/>
   </bookViews>
   <sheets>
     <sheet name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId2"/>
@@ -91,7 +91,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1582" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1484" uniqueCount="95">
   <si>
     <t xml:space="preserve">ET_adaptiveavgpool</t>
   </si>
@@ -1550,7 +1550,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19"/>
@@ -1571,12 +1571,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -1592,18 +1586,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -1621,18 +1603,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -1650,18 +1620,6 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -1679,24 +1637,15 @@
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -2302,7 +2251,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19"/>
@@ -2323,12 +2272,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -2344,18 +2287,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -2373,18 +2304,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -2402,18 +2321,6 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -2431,24 +2338,19 @@
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -2757,7 +2659,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19"/>
@@ -2778,12 +2680,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -2799,18 +2695,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -2828,18 +2712,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -2857,18 +2729,6 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -2886,24 +2746,21 @@
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -2920,7 +2777,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19"/>
@@ -2941,12 +2798,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -2962,18 +2813,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -2991,18 +2830,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -3020,18 +2847,6 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -3049,24 +2864,21 @@
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -3083,8 +2895,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
-  <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.01"/>
@@ -3104,12 +2916,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -3125,18 +2931,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -3154,18 +2948,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -3183,18 +2965,6 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -3212,24 +2982,11 @@
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -3246,7 +3003,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19"/>
@@ -3267,12 +3024,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -3288,18 +3039,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -3317,18 +3056,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -3346,18 +3073,6 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -3375,24 +3090,21 @@
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
@@ -3673,7 +3385,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19"/>
@@ -3694,12 +3406,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -3715,18 +3421,6 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -3744,18 +3438,6 @@
       <c r="E3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -3773,18 +3455,6 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -3802,24 +3472,19 @@
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-7658] Disable auto-evict in all but 4 operators
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="72"/>
   </bookViews>
   <sheets>
     <sheet name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId2"/>
@@ -469,7 +469,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -508,10 +508,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -652,7 +648,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -716,9 +712,6 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="9"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -734,10 +727,10 @@
       <c r="E2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -753,12 +746,8 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -776,10 +765,6 @@
       <c r="E4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -797,10 +782,6 @@
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
@@ -818,10 +799,6 @@
       <c r="E6" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
@@ -899,7 +876,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1398,7 +1375,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1493,7 +1470,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1585,7 +1562,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1717,7 +1694,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>7</v>
@@ -1729,7 +1706,7 @@
         <v>8</v>
       </c>
       <c r="I3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1885,7 +1862,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>7</v>
@@ -1897,7 +1874,7 @@
         <v>8</v>
       </c>
       <c r="I3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2029,7 +2006,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2140,7 +2117,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>7</v>
@@ -2152,7 +2129,7 @@
         <v>8</v>
       </c>
       <c r="I3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2286,7 +2263,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2400,7 +2377,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2496,7 +2473,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2597,7 +2574,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2694,7 +2671,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2812,7 +2789,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2930,7 +2907,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3038,7 +3015,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3160,7 +3137,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3316,7 +3293,7 @@
         <v>8</v>
       </c>
       <c r="I3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3420,7 +3397,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3536,7 +3513,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3682,7 +3659,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4144,7 +4121,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4386,7 +4363,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4403,7 +4380,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4651,7 +4628,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4758,7 +4735,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4854,7 +4831,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4961,7 +4938,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5057,7 +5034,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5283,7 +5260,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>7</v>
@@ -5295,7 +5272,7 @@
         <v>8</v>
       </c>
       <c r="I3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5436,7 +5413,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5557,7 +5534,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5654,7 +5631,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5785,7 +5762,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>7</v>
@@ -5797,7 +5774,7 @@
         <v>8</v>
       </c>
       <c r="I3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5911,7 +5888,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6007,7 +5984,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6098,7 +6075,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6115,7 +6092,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6227,7 +6204,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6324,7 +6301,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6505,7 +6482,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6619,7 +6596,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>7</v>
@@ -6631,7 +6608,7 @@
         <v>8</v>
       </c>
       <c r="I3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7345,7 +7322,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7468,7 +7445,7 @@
         <v>8</v>
       </c>
       <c r="I3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7666,7 +7643,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7807,7 +7784,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>7</v>
@@ -7819,7 +7796,7 @@
         <v>8</v>
       </c>
       <c r="I3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8016,7 +7993,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8373,7 +8350,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -8448,7 +8425,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8546,7 +8523,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8650,7 +8627,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8780,7 +8757,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8909,7 +8886,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>7</v>
@@ -8921,7 +8898,7 @@
         <v>8</v>
       </c>
       <c r="I3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9016,12 +8993,12 @@
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="14.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="13.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="13.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="6" style="0" width="8.67"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="11" t="s">
         <v>95</v>
       </c>
       <c r="B1" s="3" t="s">
@@ -9032,7 +9009,7 @@
       <c r="E1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="12"/>
+      <c r="A2" s="11"/>
       <c r="B2" s="4" t="s">
         <v>2</v>
       </c>
@@ -9047,7 +9024,7 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="12" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="0" t="s">
@@ -9345,7 +9322,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>7</v>
@@ -9357,7 +9334,7 @@
         <v>8</v>
       </c>
       <c r="I3" s="1" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[dnn-library] [SW-16407] Fix ElementSin/ElementCos/ElementNot
- Fix naming for ElementSin/ElementCos/ElementNot

- Fix implementation for sin/cos using sinf/cosf instead of Taylor
  expansion (the computation was wrong and the precision was lower
  than stated).

- Generate files with the updated IOperators.inc from Neuralizer to
  reduce one step in integrating the support. Need to merge the new
  IOperators.inc in Neuralizer.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="13" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="48" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId1"/>
@@ -20,15 +20,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_convolution3d" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_convtranspose" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_copy" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_cos" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_crossentropyloss" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_cumsum" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_dequantize" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementadd" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementcmpeq" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementcmplt" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementcmplte" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementcmpneq" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_crossentropyloss" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_cumsum" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_dequantize" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementadd" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementcmpeq" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementcmplt" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementcmplte" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementcmpneq" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementcos" sheetId="22" state="visible" r:id="rId22"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementdiv" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementerf" sheetId="24" state="visible" r:id="rId24"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementexp" sheetId="25" state="visible" r:id="rId25"/>
@@ -38,41 +38,41 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementmin" sheetId="29" state="visible" r:id="rId29"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementmul" sheetId="30" state="visible" r:id="rId30"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementneg" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementpow" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementselect" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementsub" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_embeddingbag" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_etsocgenericop" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_extracttensor" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_flip" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_frwquantizedsparselengthssum" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_frwquantizedsparselwsum" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_fullyconnected" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_gather" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_gatherranges" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_inserttensor" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_int8converter" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_intlookuptable" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_lengthsrangefill" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_lengthssum" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_lengthstoranges" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_localresponsenormalization" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_logicalnot" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_matmul" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_maxpool" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_maxpoolwithargmax" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_maxsplat" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_modulo" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_nonmaxsuppression" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_quantize" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_rescalequantized" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_resizebilinear" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_resizenearest" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_rwquantizedfullyconnected" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_rwquantizedsparselengthswsum" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_scatterdata" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_sigmoid" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_sin" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementnot" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementpow" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementselect" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementsin" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_elementsub" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_embeddingbag" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_etsocgenericop" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_extracttensor" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_flip" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_frwquantizedsparselengthssum" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_frwquantizedsparselwsum" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_fullyconnected" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_gather" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_gatherranges" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_inserttensor" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_int8converter" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_intlookuptable" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_lengthsrangefill" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_lengthssum" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_lengthstoranges" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_localresponsenormalization" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_matmul" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_maxpool" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_maxpoolwithargmax" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_maxsplat" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_modulo" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_nonmaxsuppression" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_quantize" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_rescalequantized" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_resizebilinear" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_resizenearest" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_rwquantizedfullyconnected" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_rwquantizedsparselengthswsum" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_scatterdata" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_sigmoid" sheetId="66" state="visible" r:id="rId66"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_softmax" sheetId="67" state="visible" r:id="rId67"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_spacetodepth" sheetId="68" state="visible" r:id="rId68"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_sparselengthssum" sheetId="69" state="visible" r:id="rId69"/>
@@ -1079,7 +1079,7 @@
     <col width="22.01" customWidth="1" style="13" min="1" max="1"/>
     <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
     <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
-    <col width="14.51" customWidth="1" style="13" min="6" max="6"/>
+    <col width="14.52" customWidth="1" style="13" min="6" max="6"/>
     <col width="8.67" customWidth="1" style="13" min="7" max="1025"/>
   </cols>
   <sheetData>
@@ -1444,130 +1444,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="13.01" customWidth="1" style="13" min="1" max="1"/>
-    <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
-    <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
-    <col width="16" customWidth="1" style="13" min="6" max="7"/>
-    <col width="13.01" customWidth="1" style="13" min="8" max="10"/>
-    <col width="8.67" customWidth="1" style="13" min="11" max="1025"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15" customHeight="1" s="14">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>ET_cos</t>
-        </is>
-      </c>
-      <c r="B1" s="16" t="inlineStr">
-        <is>
-          <t>BaseImpl</t>
-        </is>
-      </c>
-      <c r="F1" s="16" t="n"/>
-    </row>
-    <row r="2" ht="15" customHeight="1" s="14">
-      <c r="B2" s="17" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="C2" s="17" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="D2" s="17" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="E2" s="17" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
-      <c r="F2" s="17" t="inlineStr">
-        <is>
-          <t>dstGlobalStore</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="14">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>out0</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="14">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>in0</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="A1:A2"/>
-  </mergeCells>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
   <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
@@ -1716,7 +1592,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1839,7 +1715,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1965,7 +1841,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2109,6 +1985,255 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B1:E1"/>
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="20.99" customWidth="1" style="13" min="1" max="1"/>
+    <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
+    <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
+    <col width="16" customWidth="1" style="13" min="6" max="7"/>
+    <col width="13.01" customWidth="1" style="13" min="8" max="10"/>
+    <col width="18" customWidth="1" style="13" min="11" max="12"/>
+    <col width="13.01" customWidth="1" style="13" min="13" max="15"/>
+    <col width="8.67" customWidth="1" style="13" min="16" max="1025"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1" s="14">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>ET_elementcmpeq</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>BaseImpl</t>
+        </is>
+      </c>
+      <c r="F1" s="16" t="n"/>
+      <c r="G1" s="18" t="inlineStr">
+        <is>
+          <t>Vectorized</t>
+        </is>
+      </c>
+      <c r="K1" s="18" t="n"/>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="14">
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D2" s="17" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>evictAv</t>
+        </is>
+      </c>
+      <c r="F2" s="17" t="inlineStr">
+        <is>
+          <t>dstGlobalStore</t>
+        </is>
+      </c>
+      <c r="G2" s="19" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="H2" s="19" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I2" s="19" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="J2" s="19" t="inlineStr">
+        <is>
+          <t>evictAv</t>
+        </is>
+      </c>
+      <c r="K2" s="17" t="inlineStr">
+        <is>
+          <t>dstGlobalStore</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="14">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>out0</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="14">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>in0</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="14">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>in1</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="G1:J1"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -2139,7 +2264,7 @@
     <row r="1" ht="15" customHeight="1" s="14">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>ET_elementcmpeq</t>
+          <t>ET_elementcmplt</t>
         </is>
       </c>
       <c r="B1" s="16" t="inlineStr">
@@ -2497,7 +2622,7 @@
   <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="20.99" customWidth="1" style="13" min="1" max="1"/>
+    <col width="22.01" customWidth="1" style="13" min="1" max="1"/>
     <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
     <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
     <col width="16" customWidth="1" style="13" min="6" max="7"/>
@@ -2510,7 +2635,7 @@
     <row r="1" ht="15" customHeight="1" s="14">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>ET_elementcmplt</t>
+          <t>ET_elementcmplte</t>
         </is>
       </c>
       <c r="B1" s="16" t="inlineStr">
@@ -2746,7 +2871,7 @@
   <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="22.01" customWidth="1" style="13" min="1" max="1"/>
+    <col width="20.99" customWidth="1" style="13" min="1" max="1"/>
     <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
     <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
     <col width="16" customWidth="1" style="13" min="6" max="7"/>
@@ -2759,7 +2884,7 @@
     <row r="1" ht="15" customHeight="1" s="14">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>ET_elementcmplte</t>
+          <t>ET_elementcmpneq</t>
         </is>
       </c>
       <c r="B1" s="16" t="inlineStr">
@@ -2992,23 +3117,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="20.99" customWidth="1" style="13" min="1" max="1"/>
+    <col width="13.01" customWidth="1" style="13" min="1" max="1"/>
     <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
     <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
     <col width="16" customWidth="1" style="13" min="6" max="7"/>
     <col width="13.01" customWidth="1" style="13" min="8" max="10"/>
-    <col width="18" customWidth="1" style="13" min="11" max="12"/>
-    <col width="13.01" customWidth="1" style="13" min="13" max="15"/>
-    <col width="8.67" customWidth="1" style="13" min="16" max="1025"/>
+    <col width="8.67" customWidth="1" style="13" min="11" max="1025"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="14">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>ET_elementcmpneq</t>
+          <t>ET_elementcos</t>
         </is>
       </c>
       <c r="B1" s="16" t="inlineStr">
@@ -3017,12 +3140,6 @@
         </is>
       </c>
       <c r="F1" s="16" t="n"/>
-      <c r="G1" s="18" t="inlineStr">
-        <is>
-          <t>Vectorized</t>
-        </is>
-      </c>
-      <c r="K1" s="18" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1" s="14">
       <c r="B2" s="17" t="inlineStr">
@@ -3050,31 +3167,6 @@
           <t>dstGlobalStore</t>
         </is>
       </c>
-      <c r="G2" s="19" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="H2" s="19" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="I2" s="19" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="J2" s="19" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
-      <c r="K2" s="17" t="inlineStr">
-        <is>
-          <t>dstGlobalStore</t>
-        </is>
-      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="14">
       <c r="A3" s="15" t="inlineStr">
@@ -3103,27 +3195,6 @@
       <c r="F3" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="H3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="I3" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="J3" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="13" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="14">
       <c r="A4" s="15" t="inlineStr">
@@ -3152,81 +3223,10 @@
       <c r="F4" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="H4" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="I4" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="J4" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="14">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>in1</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="H5" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="I5" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="J5" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="13" t="n">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="G1:J1"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -3521,7 +3521,7 @@
     <col width="19" customWidth="1" style="13" min="1" max="1"/>
     <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
     <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
-    <col width="14.51" customWidth="1" style="13" min="6" max="6"/>
+    <col width="14.52" customWidth="1" style="13" min="6" max="6"/>
     <col width="8.67" customWidth="1" style="13" min="7" max="1025"/>
   </cols>
   <sheetData>
@@ -4665,6 +4665,130 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.01" customWidth="1" style="13" min="1" max="1"/>
+    <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
+    <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
+    <col width="16" customWidth="1" style="13" min="6" max="7"/>
+    <col width="13.01" customWidth="1" style="13" min="8" max="10"/>
+    <col width="8.67" customWidth="1" style="13" min="11" max="1025"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1" s="14">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>ET_elementnot</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>BaseImpl</t>
+        </is>
+      </c>
+      <c r="F1" s="16" t="n"/>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="14">
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D2" s="17" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>evictAv</t>
+        </is>
+      </c>
+      <c r="F2" s="17" t="inlineStr">
+        <is>
+          <t>dstGlobalStore</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="14">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>out0</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="14">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>in0</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
@@ -4811,7 +4935,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4993,7 +5117,131 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.01" customWidth="1" style="13" min="1" max="1"/>
+    <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
+    <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
+    <col width="16" customWidth="1" style="13" min="6" max="7"/>
+    <col width="13.01" customWidth="1" style="13" min="8" max="10"/>
+    <col width="8.67" customWidth="1" style="13" min="11" max="1025"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1" s="14">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>ET_elementsin</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>BaseImpl</t>
+        </is>
+      </c>
+      <c r="F1" s="16" t="n"/>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="14">
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D2" s="17" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>evictAv</t>
+        </is>
+      </c>
+      <c r="F2" s="17" t="inlineStr">
+        <is>
+          <t>dstGlobalStore</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="14">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>out0</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="14">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>in0</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5145,7 +5393,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5633,7 +5881,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5762,7 +6010,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5880,311 +6128,6 @@
   <mergeCells count="3">
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="G1:J1"/>
-    <mergeCell ref="A1:A2"/>
-  </mergeCells>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="13.01" customWidth="1" style="13" min="1" max="1"/>
-    <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
-    <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
-    <col width="15.34" customWidth="1" style="13" min="6" max="6"/>
-    <col width="8.67" customWidth="1" style="13" min="7" max="1025"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15" customHeight="1" s="14">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>ET_flip</t>
-        </is>
-      </c>
-      <c r="B1" s="16" t="inlineStr">
-        <is>
-          <t>BaseImpl</t>
-        </is>
-      </c>
-      <c r="F1" s="16" t="n"/>
-    </row>
-    <row r="2" ht="15" customHeight="1" s="14">
-      <c r="B2" s="17" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="C2" s="17" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="D2" s="17" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="E2" s="17" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
-      <c r="F2" s="17" t="inlineStr">
-        <is>
-          <t>dstGlobalStore</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="14">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>out0</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="14">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>in0</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="A1:A2"/>
-  </mergeCells>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="45.99" customWidth="1" style="13" min="1" max="1"/>
-    <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
-    <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
-    <col width="16" customWidth="1" style="13" min="6" max="7"/>
-    <col width="13.01" customWidth="1" style="13" min="8" max="10"/>
-    <col width="18" customWidth="1" style="13" min="11" max="11"/>
-    <col width="13.01" customWidth="1" style="13" min="12" max="14"/>
-    <col width="8.67" customWidth="1" style="13" min="15" max="1025"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15" customHeight="1" s="14">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>ET_fusedrowwisequantizedsparselengthssum</t>
-        </is>
-      </c>
-      <c r="B1" s="16" t="inlineStr">
-        <is>
-          <t>BaseImpl</t>
-        </is>
-      </c>
-      <c r="F1" s="16" t="n"/>
-    </row>
-    <row r="2" ht="15" customHeight="1" s="14">
-      <c r="B2" s="17" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="C2" s="17" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="D2" s="17" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="E2" s="17" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
-      <c r="F2" s="17" t="inlineStr">
-        <is>
-          <t>dstGlobalStore</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="14">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>out0</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="14">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>in0</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="14">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>in1</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="14">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>in2</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B1:E1"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -6352,23 +6295,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="53.99" customWidth="1" style="13" min="1" max="1"/>
+    <col width="13.01" customWidth="1" style="13" min="1" max="1"/>
     <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
     <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
-    <col width="16" customWidth="1" style="13" min="6" max="7"/>
-    <col width="13.01" customWidth="1" style="13" min="8" max="10"/>
-    <col width="18" customWidth="1" style="13" min="11" max="11"/>
-    <col width="13.01" customWidth="1" style="13" min="12" max="14"/>
-    <col width="8.67" customWidth="1" style="13" min="15" max="1025"/>
+    <col width="15.34" customWidth="1" style="13" min="6" max="6"/>
+    <col width="8.67" customWidth="1" style="13" min="7" max="1025"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="14">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>ET_fusedrowwisequantizedsparselengthsweightedsum</t>
+          <t>ET_flip</t>
         </is>
       </c>
       <c r="B1" s="16" t="inlineStr">
@@ -6458,90 +6398,6 @@
         <v>0</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="14">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>in1</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="14">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>in2</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="14">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>in3</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6565,6 +6421,398 @@
   <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
+    <col width="45.99" customWidth="1" style="13" min="1" max="1"/>
+    <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
+    <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
+    <col width="16" customWidth="1" style="13" min="6" max="7"/>
+    <col width="13.01" customWidth="1" style="13" min="8" max="10"/>
+    <col width="18" customWidth="1" style="13" min="11" max="11"/>
+    <col width="13.01" customWidth="1" style="13" min="12" max="14"/>
+    <col width="8.67" customWidth="1" style="13" min="15" max="1025"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1" s="14">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>ET_fusedrowwisequantizedsparselengthssum</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>BaseImpl</t>
+        </is>
+      </c>
+      <c r="F1" s="16" t="n"/>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="14">
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D2" s="17" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>evictAv</t>
+        </is>
+      </c>
+      <c r="F2" s="17" t="inlineStr">
+        <is>
+          <t>dstGlobalStore</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="14">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>out0</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="14">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>in0</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="14">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>in1</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="14">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>in2</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="53.99" customWidth="1" style="13" min="1" max="1"/>
+    <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
+    <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
+    <col width="16" customWidth="1" style="13" min="6" max="7"/>
+    <col width="13.01" customWidth="1" style="13" min="8" max="10"/>
+    <col width="18" customWidth="1" style="13" min="11" max="11"/>
+    <col width="13.01" customWidth="1" style="13" min="12" max="14"/>
+    <col width="8.67" customWidth="1" style="13" min="15" max="1025"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1" s="14">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>ET_fusedrowwisequantizedsparselengthsweightedsum</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>BaseImpl</t>
+        </is>
+      </c>
+      <c r="F1" s="16" t="n"/>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="14">
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D2" s="17" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>evictAv</t>
+        </is>
+      </c>
+      <c r="F2" s="17" t="inlineStr">
+        <is>
+          <t>dstGlobalStore</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="14">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>out0</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="14">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>in0</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="14">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>in1</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="14">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>in2</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1" s="14">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>in3</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
     <col width="23.01" customWidth="1" style="13" min="1" max="1"/>
     <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
     <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
@@ -6738,7 +6986,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6892,7 +7140,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7074,7 +7322,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7258,283 +7506,6 @@
         <v>0</v>
       </c>
       <c r="K4" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="G1:J1"/>
-    <mergeCell ref="A1:A2"/>
-  </mergeCells>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="22.01" customWidth="1" style="13" min="1" max="1"/>
-    <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
-    <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
-    <col width="15" customWidth="1" style="13" min="6" max="6"/>
-    <col width="8.67" customWidth="1" style="13" min="7" max="1025"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15" customHeight="1" s="14">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>ET_int8converter</t>
-        </is>
-      </c>
-      <c r="B1" s="16" t="inlineStr">
-        <is>
-          <t>BaseImpl</t>
-        </is>
-      </c>
-      <c r="F1" s="16" t="n"/>
-    </row>
-    <row r="2" ht="15" customHeight="1" s="14">
-      <c r="B2" s="17" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="C2" s="17" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="D2" s="17" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="E2" s="17" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
-      <c r="F2" s="17" t="inlineStr">
-        <is>
-          <t>dstGlobalStore</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="14">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>out0</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="14">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>in0</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="A1:A2"/>
-  </mergeCells>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:J5"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="23.01" customWidth="1" style="13" min="1" max="1"/>
-    <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
-    <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
-    <col width="16" customWidth="1" style="13" min="6" max="7"/>
-    <col width="13.01" customWidth="1" style="13" min="8" max="10"/>
-    <col width="8.67" customWidth="1" style="13" min="11" max="1025"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15" customHeight="1" s="14">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>ET_intlookuptable</t>
-        </is>
-      </c>
-      <c r="B1" s="16" t="inlineStr">
-        <is>
-          <t>BaseImpl</t>
-        </is>
-      </c>
-      <c r="F1" s="16" t="n"/>
-      <c r="G1" s="13" t="n"/>
-    </row>
-    <row r="2" ht="15" customHeight="1" s="14">
-      <c r="B2" s="17" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="C2" s="17" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="D2" s="17" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="E2" s="17" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
-      <c r="F2" s="17" t="inlineStr">
-        <is>
-          <t>dstGlobalStore</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="14">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>out0</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="14">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>in0</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="14">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>in1</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7559,17 +7530,17 @@
   <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="25" customWidth="1" style="13" min="1" max="1"/>
+    <col width="22.01" customWidth="1" style="13" min="1" max="1"/>
     <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
     <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
-    <col width="16.33" customWidth="1" style="13" min="6" max="6"/>
+    <col width="15" customWidth="1" style="13" min="6" max="6"/>
     <col width="8.67" customWidth="1" style="13" min="7" max="1025"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="14">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>ET_lengthsrangefill</t>
+          <t>ET_int8converter</t>
         </is>
       </c>
       <c r="B1" s="16" t="inlineStr">
@@ -7682,7 +7653,7 @@
   <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="19" customWidth="1" style="13" min="1" max="1"/>
+    <col width="23.01" customWidth="1" style="13" min="1" max="1"/>
     <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
     <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
     <col width="16" customWidth="1" style="13" min="6" max="7"/>
@@ -7693,7 +7664,7 @@
     <row r="1" ht="15" customHeight="1" s="14">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>ET_lengthssum</t>
+          <t>ET_intlookuptable</t>
         </is>
       </c>
       <c r="B1" s="16" t="inlineStr">
@@ -7833,21 +7804,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="24" customWidth="1" style="13" min="1" max="1"/>
+    <col width="25" customWidth="1" style="13" min="1" max="1"/>
     <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
     <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
-    <col width="16" customWidth="1" style="13" min="6" max="7"/>
-    <col width="13.01" customWidth="1" style="13" min="8" max="10"/>
-    <col width="8.67" customWidth="1" style="13" min="11" max="1025"/>
+    <col width="16.33" customWidth="1" style="13" min="6" max="6"/>
+    <col width="8.67" customWidth="1" style="13" min="7" max="1025"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="14">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>ET_lengthstoranges</t>
+          <t>ET_lengthsrangefill</t>
         </is>
       </c>
       <c r="B1" s="16" t="inlineStr">
@@ -7856,7 +7826,6 @@
         </is>
       </c>
       <c r="F1" s="16" t="n"/>
-      <c r="G1" s="13" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1" s="14">
       <c r="B2" s="17" t="inlineStr">
@@ -7942,9 +7911,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="G1:J1"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -8084,23 +8052,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="35" customWidth="1" style="13" min="1" max="1"/>
+    <col width="19" customWidth="1" style="13" min="1" max="1"/>
     <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
     <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
     <col width="16" customWidth="1" style="13" min="6" max="7"/>
     <col width="13.01" customWidth="1" style="13" min="8" max="10"/>
-    <col width="18" customWidth="1" style="13" min="11" max="12"/>
-    <col width="13.01" customWidth="1" style="13" min="13" max="15"/>
-    <col width="8.67" customWidth="1" style="13" min="16" max="1025"/>
+    <col width="8.67" customWidth="1" style="13" min="11" max="1025"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="14">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>ET_localresponsenormalization</t>
+          <t>ET_lengthssum</t>
         </is>
       </c>
       <c r="B1" s="16" t="inlineStr">
@@ -8109,12 +8075,7 @@
         </is>
       </c>
       <c r="F1" s="16" t="n"/>
-      <c r="G1" s="18" t="inlineStr">
-        <is>
-          <t>Vectorized</t>
-        </is>
-      </c>
-      <c r="K1" s="18" t="n"/>
+      <c r="G1" s="13" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1" s="14">
       <c r="B2" s="17" t="inlineStr">
@@ -8142,31 +8103,6 @@
           <t>dstGlobalStore</t>
         </is>
       </c>
-      <c r="G2" s="19" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="H2" s="19" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="I2" s="19" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="J2" s="19" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
-      <c r="K2" s="18" t="inlineStr">
-        <is>
-          <t>dstGlobalStore</t>
-        </is>
-      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="14">
       <c r="A3" s="15" t="inlineStr">
@@ -8195,42 +8131,21 @@
       <c r="F3" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="H3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="I3" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="J3" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="13" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="14">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>out1</t>
+          <t>in0</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>dirty</t>
+          <t>clean</t>
         </is>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>dirty</t>
+          <t>clean</t>
         </is>
       </c>
       <c r="D4" s="13" t="inlineStr">
@@ -8242,34 +8157,13 @@
         <v>0</v>
       </c>
       <c r="F4" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="H4" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="I4" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="J4" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="13" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="14">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>in0</t>
+          <t>in1</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
@@ -8291,27 +8185,6 @@
         <v>0</v>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="H5" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="I5" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="J5" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8333,10 +8206,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="13.01" customWidth="1" style="13" min="1" max="1"/>
+    <col width="24" customWidth="1" style="13" min="1" max="1"/>
     <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
     <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
     <col width="16" customWidth="1" style="13" min="6" max="7"/>
@@ -8347,7 +8220,7 @@
     <row r="1" ht="15" customHeight="1" s="14">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>ET_logicalnot</t>
+          <t>ET_lengthstoranges</t>
         </is>
       </c>
       <c r="B1" s="16" t="inlineStr">
@@ -8356,6 +8229,7 @@
         </is>
       </c>
       <c r="F1" s="16" t="n"/>
+      <c r="G1" s="13" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1" s="14">
       <c r="B2" s="17" t="inlineStr">
@@ -8441,8 +8315,9 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="B1:E1"/>
+    <mergeCell ref="G1:J1"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -8452,6 +8327,255 @@
 </file>
 
 <file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="35" customWidth="1" style="13" min="1" max="1"/>
+    <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
+    <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
+    <col width="16" customWidth="1" style="13" min="6" max="7"/>
+    <col width="13.01" customWidth="1" style="13" min="8" max="10"/>
+    <col width="18" customWidth="1" style="13" min="11" max="12"/>
+    <col width="13.01" customWidth="1" style="13" min="13" max="15"/>
+    <col width="8.67" customWidth="1" style="13" min="16" max="1025"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1" s="14">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>ET_localresponsenormalization</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>BaseImpl</t>
+        </is>
+      </c>
+      <c r="F1" s="16" t="n"/>
+      <c r="G1" s="18" t="inlineStr">
+        <is>
+          <t>Vectorized</t>
+        </is>
+      </c>
+      <c r="K1" s="18" t="n"/>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="14">
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D2" s="17" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>evictAv</t>
+        </is>
+      </c>
+      <c r="F2" s="17" t="inlineStr">
+        <is>
+          <t>dstGlobalStore</t>
+        </is>
+      </c>
+      <c r="G2" s="19" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="H2" s="19" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="I2" s="19" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="J2" s="19" t="inlineStr">
+        <is>
+          <t>evictAv</t>
+        </is>
+      </c>
+      <c r="K2" s="18" t="inlineStr">
+        <is>
+          <t>dstGlobalStore</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="14">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>out0</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="14">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>out1</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="14">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>in0</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="G1:J1"/>
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8605,7 +8729,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8731,7 +8855,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8885,7 +9009,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9087,7 +9211,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9213,7 +9337,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9392,7 +9516,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9413,132 +9537,6 @@
       <c r="A1" s="15" t="inlineStr">
         <is>
           <t>ET_quantize</t>
-        </is>
-      </c>
-      <c r="B1" s="16" t="inlineStr">
-        <is>
-          <t>BaseImpl</t>
-        </is>
-      </c>
-      <c r="F1" s="16" t="n"/>
-      <c r="G1" s="13" t="n"/>
-    </row>
-    <row r="2" ht="15" customHeight="1" s="14">
-      <c r="B2" s="17" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="C2" s="17" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="D2" s="17" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="E2" s="17" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
-      <c r="F2" s="17" t="inlineStr">
-        <is>
-          <t>dstGlobalStore</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="14">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>out0</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="14">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>in0</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="G1:J1"/>
-    <mergeCell ref="A1:A2"/>
-  </mergeCells>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:J4"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="25" customWidth="1" style="13" min="1" max="1"/>
-    <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
-    <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
-    <col width="16" customWidth="1" style="13" min="6" max="7"/>
-    <col width="13.01" customWidth="1" style="13" min="8" max="10"/>
-    <col width="8.67" customWidth="1" style="13" min="11" max="1025"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15" customHeight="1" s="14">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>ET_rescalequantized</t>
         </is>
       </c>
       <c r="B1" s="16" t="inlineStr">
@@ -9772,20 +9770,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="23.01" customWidth="1" style="13" min="1" max="1"/>
+    <col width="25" customWidth="1" style="13" min="1" max="1"/>
     <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
     <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
-    <col width="15" customWidth="1" style="13" min="6" max="6"/>
-    <col width="8.67" customWidth="1" style="13" min="7" max="1025"/>
+    <col width="16" customWidth="1" style="13" min="6" max="7"/>
+    <col width="13.01" customWidth="1" style="13" min="8" max="10"/>
+    <col width="8.67" customWidth="1" style="13" min="11" max="1025"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="14">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>ET_resizebilinear</t>
+          <t>ET_rescalequantized</t>
         </is>
       </c>
       <c r="B1" s="16" t="inlineStr">
@@ -9794,6 +9793,7 @@
         </is>
       </c>
       <c r="F1" s="16" t="n"/>
+      <c r="G1" s="13" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1" s="14">
       <c r="B2" s="17" t="inlineStr">
@@ -9879,8 +9879,9 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="B1:E1"/>
+    <mergeCell ref="G1:J1"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -9898,17 +9899,17 @@
   <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="22.01" customWidth="1" style="13" min="1" max="1"/>
+    <col width="23.01" customWidth="1" style="13" min="1" max="1"/>
     <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
     <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
-    <col width="14.83" customWidth="1" style="13" min="6" max="6"/>
+    <col width="15" customWidth="1" style="13" min="6" max="6"/>
     <col width="8.67" customWidth="1" style="13" min="7" max="1025"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="14">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>ET_resizenearest</t>
+          <t>ET_resizebilinear</t>
         </is>
       </c>
       <c r="B1" s="16" t="inlineStr">
@@ -10013,6 +10014,129 @@
 </file>
 
 <file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="22.01" customWidth="1" style="13" min="1" max="1"/>
+    <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
+    <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
+    <col width="14.83" customWidth="1" style="13" min="6" max="6"/>
+    <col width="8.67" customWidth="1" style="13" min="7" max="1025"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1" s="14">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>ET_resizenearest</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>BaseImpl</t>
+        </is>
+      </c>
+      <c r="F1" s="16" t="n"/>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="14">
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D2" s="17" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>evictAv</t>
+        </is>
+      </c>
+      <c r="F2" s="17" t="inlineStr">
+        <is>
+          <t>dstGlobalStore</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="14">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>out0</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="14">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>in0</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10410,7 +10534,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10855,7 +10979,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11006,7 +11130,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11126,130 +11250,6 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B1:F1"/>
-    <mergeCell ref="A1:A2"/>
-  </mergeCells>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="13.01" customWidth="1" style="13" min="1" max="1"/>
-    <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
-    <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
-    <col width="16" customWidth="1" style="13" min="6" max="7"/>
-    <col width="13.01" customWidth="1" style="13" min="8" max="10"/>
-    <col width="8.67" customWidth="1" style="13" min="11" max="1025"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15" customHeight="1" s="14">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>ET_sin</t>
-        </is>
-      </c>
-      <c r="B1" s="16" t="inlineStr">
-        <is>
-          <t>BaseImpl</t>
-        </is>
-      </c>
-      <c r="F1" s="16" t="n"/>
-    </row>
-    <row r="2" ht="15" customHeight="1" s="14">
-      <c r="B2" s="17" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="C2" s="17" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="D2" s="17" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="E2" s="17" t="inlineStr">
-        <is>
-          <t>evictAv</t>
-        </is>
-      </c>
-      <c r="F2" s="17" t="inlineStr">
-        <is>
-          <t>dstGlobalStore</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="14">
-      <c r="A3" s="15" t="inlineStr">
-        <is>
-          <t>out0</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>dirty</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="14">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>in0</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>untouched</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B1:E1"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-16351] Add empty implementation for Trilu in dnn library
- Add empty implementation for Trilu in dnn library.

- Add Upper boolean parameter for Trilu.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="48" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="76" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId1"/>
@@ -86,7 +86,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_topk" sheetId="77" state="visible" r:id="rId77"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_touch" sheetId="78" state="visible" r:id="rId78"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_transpose" sheetId="79" state="visible" r:id="rId79"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INFORMATION" sheetId="80" state="visible" r:id="rId80"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ET_trilu" sheetId="80" state="visible" r:id="rId80"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INFORMATION" sheetId="81" state="visible" r:id="rId81"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -13986,6 +13987,158 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="19" customWidth="1" style="13" min="1" max="1"/>
+    <col width="14.01" customWidth="1" style="13" min="2" max="2"/>
+    <col width="13.01" customWidth="1" style="13" min="3" max="5"/>
+    <col width="18" customWidth="1" style="13" min="6" max="7"/>
+    <col width="13.01" customWidth="1" style="13" min="8" max="10"/>
+    <col width="8.67" customWidth="1" style="13" min="11" max="1025"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1" s="14">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>ET_trilu</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>BaseImpl</t>
+        </is>
+      </c>
+      <c r="F1" s="16" t="n"/>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="14">
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="D2" s="17" t="inlineStr">
+        <is>
+          <t>CB</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>evictAv</t>
+        </is>
+      </c>
+      <c r="F2" s="17" t="inlineStr">
+        <is>
+          <t>dstGlobalStore</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="14">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>out0</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>dirty</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="14">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>in0</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="14">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>in1</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>untouched</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
   <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="13" zeroHeight="0" outlineLevelRow="0"/>
   <cols>

</xml_diff>

<commit_message>
[dnn-library] [SW-20442] Get rid of single-threaded DequantizeNBitsColumnBlocksInst.
The multi-threaded implementation is the only one left.
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -106,7 +106,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1965" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1929" uniqueCount="113">
   <si>
     <t xml:space="preserve">ET_adaptiveavgpool</t>
   </si>
@@ -1853,16 +1853,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16380" style="0" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1875,12 +1873,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="G1" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -1899,21 +1891,6 @@
       <c r="F2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="K2" s="7" t="s">
-        <v>6</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -1934,21 +1911,6 @@
       <c r="F3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -1969,21 +1931,6 @@
       <c r="F4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -2004,21 +1951,6 @@
       <c r="F5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
@@ -2039,27 +1971,11 @@
       <c r="F6" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="G1:J1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2076,16 +1992,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="1" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16380" style="0" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2098,12 +2012,6 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="G1" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -2122,21 +2030,6 @@
       <c r="F2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="K2" s="7" t="s">
-        <v>6</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -2157,21 +2050,6 @@
       <c r="F3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -2192,21 +2070,6 @@
       <c r="F4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -2227,21 +2090,6 @@
       <c r="F5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
@@ -2262,27 +2110,11 @@
       <c r="F6" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="1" t="n">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="G1:J1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
[dnn-library] [SW-22172] Optimize resize nearest when channel upscaling is 1
</commit_message>
<xml_diff>
--- a/dnn-library/scripts/cacheState.xlsx
+++ b/dnn-library/scripts/cacheState.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="67"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="68"/>
   </bookViews>
   <sheets>
     <sheet name="ET_adaptiveavgpool" sheetId="1" state="visible" r:id="rId3"/>
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1972" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1984" uniqueCount="116">
   <si>
     <t xml:space="preserve">ET_adaptiveavgpool</t>
   </si>
@@ -386,6 +386,9 @@
   </si>
   <si>
     <t xml:space="preserve">ET_resizenearest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NoUpscaleC</t>
   </si>
   <si>
     <t xml:space="preserve">ET_rowwisequantizedfullyconnected</t>
@@ -9429,13 +9432,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="12" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="1" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="17.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="13.63"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9456,6 +9461,13 @@
       <c r="I1" s="6"/>
       <c r="J1" s="6"/>
       <c r="K1" s="12"/>
+      <c r="L1" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
+      <c r="O1" s="3"/>
+      <c r="P1" s="11"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -9489,6 +9501,21 @@
       <c r="K2" s="7" t="s">
         <v>6</v>
       </c>
+      <c r="L2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="O2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
@@ -9524,6 +9551,21 @@
       <c r="K3" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="L3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="O3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -9559,12 +9601,28 @@
       <c r="K4" s="1" t="n">
         <v>0</v>
       </c>
+      <c r="L4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="O4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="G1:J1"/>
+    <mergeCell ref="L1:O1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -9742,7 +9800,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -10037,7 +10095,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -10364,7 +10422,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -10484,7 +10542,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -10587,7 +10645,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -10739,7 +10797,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -10840,7 +10898,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -11063,7 +11121,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -11323,7 +11381,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -11448,7 +11506,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -11832,7 +11890,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -11911,7 +11969,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -12011,7 +12069,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -12113,7 +12171,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -12213,7 +12271,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -12337,7 +12395,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -12370,13 +12428,13 @@
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>0</v>
@@ -12419,7 +12477,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -12572,7 +12630,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
@@ -12688,17 +12746,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>